<commit_message>
Cap nhat du lieu - 12/05/2026 16:12
</commit_message>
<xml_diff>
--- a/HangMuc.xlsx
+++ b/HangMuc.xlsx
@@ -1677,9 +1677,9 @@
       <c r="F5" s="39" t="inlineStr"/>
       <c r="G5" s="40" t="inlineStr">
         <is>
-          <t>- KC: 3/2025
-- HT: 6/2025
-- QT: 7/2025</t>
+          <t>- KC: 3/2026
+- HT: 6/2026
+- QT: 7/2026</t>
         </is>
       </c>
       <c r="H5" s="42" t="n">

</xml_diff>

<commit_message>
Cap nhat du lieu - 15/05/2026 11:45
</commit_message>
<xml_diff>
--- a/HangMuc.xlsx
+++ b/HangMuc.xlsx
@@ -1254,22 +1254,22 @@
     <col width="8" customWidth="1" style="2" min="6" max="6"/>
     <col width="20" customWidth="1" style="2" min="7" max="7"/>
     <col width="20" customWidth="1" style="1" min="8" max="8"/>
-    <col width="20" customWidth="1" style="2" min="9" max="9"/>
-    <col width="13" customWidth="1" style="2" min="10" max="10"/>
+    <col width="34" customWidth="1" style="2" min="9" max="9"/>
+    <col width="16" customWidth="1" style="2" min="10" max="10"/>
     <col width="17" customWidth="1" style="1" min="11" max="11"/>
     <col width="21" customWidth="1" style="2" min="12" max="12"/>
     <col width="17" customWidth="1" style="2" min="13" max="13"/>
     <col width="20" customWidth="1" style="1" min="14" max="14"/>
     <col width="17" customWidth="1" style="1" min="15" max="15"/>
-    <col width="20" customWidth="1" style="2" min="16" max="16"/>
+    <col width="32" customWidth="1" style="2" min="16" max="16"/>
     <col width="17" customWidth="1" style="2" min="17" max="19"/>
-    <col width="23" customWidth="1" min="18" max="18"/>
+    <col width="27" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="20" customWidth="1" style="1" min="20" max="20"/>
     <col width="17" customWidth="1" style="1" min="21" max="23"/>
     <col width="23" customWidth="1" min="22" max="22"/>
     <col width="19" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" style="2" min="24" max="24"/>
+    <col width="80" customWidth="1" style="2" min="24" max="24"/>
     <col width="17" customWidth="1" style="2" min="25" max="25"/>
     <col width="11" customWidth="1" style="2" min="26" max="26"/>
     <col width="9" customWidth="1" style="2" min="27" max="27"/>
@@ -1588,14 +1588,14 @@
       </c>
       <c r="I4" s="32" t="inlineStr"/>
       <c r="J4" s="35" t="n">
-        <v>0</v>
+        <v>13254</v>
       </c>
       <c r="K4" s="35" t="n">
-        <v>12552889759</v>
+        <v>9720</v>
       </c>
       <c r="L4" s="32" t="inlineStr"/>
       <c r="M4" s="35" t="n">
-        <v>0</v>
+        <v>11333</v>
       </c>
       <c r="N4" s="32" t="inlineStr"/>
       <c r="O4" s="35" t="n">
@@ -1603,11 +1603,11 @@
       </c>
       <c r="P4" s="32" t="inlineStr"/>
       <c r="Q4" s="35" t="n">
-        <v>11333808687</v>
+        <v>9368</v>
       </c>
       <c r="R4" s="32" t="inlineStr"/>
       <c r="S4" s="35" t="n">
-        <v>0</v>
+        <v>9368</v>
       </c>
       <c r="T4" s="32" t="inlineStr"/>
       <c r="U4" s="35" t="n">
@@ -1685,16 +1685,24 @@
       <c r="H5" s="42" t="n">
         <v>12552889759</v>
       </c>
-      <c r="I5" s="39" t="inlineStr"/>
+      <c r="I5" s="39" t="inlineStr">
+        <is>
+          <t>111/QĐ_PCVT, ngày 29/03/2026</t>
+        </is>
+      </c>
       <c r="J5" s="42" t="n">
-        <v>0</v>
+        <v>13254</v>
       </c>
       <c r="K5" s="42" t="n">
-        <v>12552889759</v>
-      </c>
-      <c r="L5" s="39" t="inlineStr"/>
+        <v>9720</v>
+      </c>
+      <c r="L5" s="39" t="inlineStr">
+        <is>
+          <t>115/QĐ-PCVT</t>
+        </is>
+      </c>
       <c r="M5" s="42" t="n">
-        <v>0</v>
+        <v>11333</v>
       </c>
       <c r="N5" s="39" t="inlineStr"/>
       <c r="O5" s="42" t="n">
@@ -1702,15 +1710,19 @@
       </c>
       <c r="P5" s="39" t="inlineStr">
         <is>
-          <t>115/QĐ-PCVT</t>
+          <t>1292/TM-PCVT, ngày 26/03/2026</t>
         </is>
       </c>
       <c r="Q5" s="42" t="n">
-        <v>11333808687</v>
-      </c>
-      <c r="R5" s="39" t="inlineStr"/>
+        <v>9368</v>
+      </c>
+      <c r="R5" s="39" t="inlineStr">
+        <is>
+          <t>11-2026/HĐXL/LDLTQV-PCVT</t>
+        </is>
+      </c>
       <c r="S5" s="42" t="n">
-        <v>0</v>
+        <v>9368</v>
       </c>
       <c r="T5" s="39" t="inlineStr"/>
       <c r="U5" s="42" t="n">
@@ -1720,8 +1732,16 @@
       <c r="W5" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="X5" s="39" t="inlineStr"/>
-      <c r="Y5" s="39" t="inlineStr"/>
+      <c r="X5" s="39" t="inlineStr">
+        <is>
+          <t>LIÊN DANH CÔNG TY TNHH LẠC THÀNH VÀ CÔNG TY CỔ PHẦN DỊCH VỤ XÂY DỰNG QUANG VŨ</t>
+        </is>
+      </c>
+      <c r="Y5" s="39" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
       <c r="Z5" s="43" t="n">
         <v>0</v>
       </c>
@@ -1767,26 +1787,26 @@
       </c>
       <c r="I6" s="32" t="inlineStr"/>
       <c r="J6" s="35" t="n">
-        <v>0</v>
+        <v>3311634663</v>
       </c>
       <c r="K6" s="35" t="n">
-        <v>3765771568</v>
+        <v>14508</v>
       </c>
       <c r="L6" s="32" t="inlineStr"/>
       <c r="M6" s="35" t="n">
-        <v>0</v>
+        <v>2579</v>
       </c>
       <c r="N6" s="32" t="inlineStr"/>
       <c r="O6" s="35" t="n">
-        <v>0</v>
+        <v>11705</v>
       </c>
       <c r="P6" s="32" t="inlineStr"/>
       <c r="Q6" s="35" t="n">
-        <v>0</v>
+        <v>2412</v>
       </c>
       <c r="R6" s="32" t="inlineStr"/>
       <c r="S6" s="35" t="n">
-        <v>0</v>
+        <v>2412</v>
       </c>
       <c r="T6" s="32" t="inlineStr"/>
       <c r="U6" s="35" t="n">
@@ -1855,20 +1875,28 @@
       <c r="H7" s="42" t="n">
         <v>13650367159</v>
       </c>
-      <c r="I7" s="39" t="inlineStr"/>
+      <c r="I7" s="39" t="inlineStr">
+        <is>
+          <t>01/PAKT-QLHTĐĐ, ngày 15/10/2025</t>
+        </is>
+      </c>
       <c r="J7" s="42" t="n">
-        <v>0</v>
+        <v>13650</v>
       </c>
       <c r="K7" s="42" t="n">
-        <v>3765771568</v>
+        <v>11840</v>
       </c>
       <c r="L7" s="39" t="inlineStr"/>
       <c r="M7" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="39" t="inlineStr"/>
+      <c r="N7" s="39" t="inlineStr">
+        <is>
+          <t>07/QĐ-PCVT</t>
+        </is>
+      </c>
       <c r="O7" s="42" t="n">
-        <v>0</v>
+        <v>11705</v>
       </c>
       <c r="P7" s="39" t="inlineStr"/>
       <c r="Q7" s="42" t="n">
@@ -1886,8 +1914,16 @@
       <c r="W7" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="X7" s="39" t="inlineStr"/>
-      <c r="Y7" s="39" t="inlineStr"/>
+      <c r="X7" s="39" t="inlineStr">
+        <is>
+          <t>Công ty Điện lực Vũng Tàu</t>
+        </is>
+      </c>
+      <c r="Y7" s="39" t="inlineStr">
+        <is>
+          <t>27/01/2026</t>
+        </is>
+      </c>
       <c r="Z7" s="43" t="n">
         <v>0</v>
       </c>
@@ -1942,7 +1978,7 @@
       <c r="F8" s="39" t="inlineStr"/>
       <c r="G8" s="40" t="inlineStr">
         <is>
-          <t>- KC: T3/2026
+          <t>- KC: 3/2026
 - HT: 6/2026
 - QT: 7/2026</t>
         </is>
@@ -1950,28 +1986,44 @@
       <c r="H8" s="42" t="n">
         <v>3765771568</v>
       </c>
-      <c r="I8" s="39" t="inlineStr"/>
+      <c r="I8" s="39" t="inlineStr">
+        <is>
+          <t>129/QĐ-PCVT, ngày 12/03/2026</t>
+        </is>
+      </c>
       <c r="J8" s="42" t="n">
-        <v>0</v>
+        <v>3311621013</v>
       </c>
       <c r="K8" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="39" t="inlineStr"/>
+        <v>2668</v>
+      </c>
+      <c r="L8" s="39" t="inlineStr">
+        <is>
+          <t>161/QĐ-PCVT</t>
+        </is>
+      </c>
       <c r="M8" s="42" t="n">
-        <v>0</v>
+        <v>2579</v>
       </c>
       <c r="N8" s="39" t="inlineStr"/>
       <c r="O8" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="P8" s="39" t="inlineStr"/>
+      <c r="P8" s="39" t="inlineStr">
+        <is>
+          <t>166/QĐ-PCVT, ngày 26/03/2026</t>
+        </is>
+      </c>
       <c r="Q8" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="39" t="inlineStr"/>
+        <v>2412</v>
+      </c>
+      <c r="R8" s="39" t="inlineStr">
+        <is>
+          <t>1313/HĐ-PCVT</t>
+        </is>
+      </c>
       <c r="S8" s="42" t="n">
-        <v>0</v>
+        <v>2412</v>
       </c>
       <c r="T8" s="39" t="inlineStr"/>
       <c r="U8" s="42" t="n">
@@ -1981,8 +2033,16 @@
       <c r="W8" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="X8" s="39" t="inlineStr"/>
-      <c r="Y8" s="39" t="inlineStr"/>
+      <c r="X8" s="39" t="inlineStr">
+        <is>
+          <t>CHI NHÁNH TỔNG CÔNG TY ĐIỆN LỰC TPHCM TNHH – CÔNG TY DỊCH VỤ ĐIỆN LỰC TPHCM</t>
+        </is>
+      </c>
+      <c r="Y8" s="39" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
       <c r="Z8" s="43" t="n">
         <v>0</v>
       </c>
@@ -2031,7 +2091,7 @@
         <v>0</v>
       </c>
       <c r="K9" s="35" t="n">
-        <v>1590994000</v>
+        <v>1125</v>
       </c>
       <c r="L9" s="32" t="inlineStr"/>
       <c r="M9" s="35" t="n">
@@ -2130,7 +2190,7 @@
         <v>0</v>
       </c>
       <c r="K10" s="42" t="n">
-        <v>1590994000</v>
+        <v>1125</v>
       </c>
       <c r="L10" s="39" t="inlineStr"/>
       <c r="M10" s="42" t="n">
@@ -2156,7 +2216,11 @@
       <c r="W10" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="X10" s="39" t="inlineStr"/>
+      <c r="X10" s="39" t="inlineStr">
+        <is>
+          <t>Công ty điện lực Vũng Tàu</t>
+        </is>
+      </c>
       <c r="Y10" s="39" t="inlineStr"/>
       <c r="Z10" s="43" t="n">
         <v>0</v>
@@ -2203,10 +2267,10 @@
       </c>
       <c r="I11" s="32" t="inlineStr"/>
       <c r="J11" s="35" t="n">
-        <v>0</v>
+        <v>523</v>
       </c>
       <c r="K11" s="35" t="n">
-        <v>527000000</v>
+        <v>440</v>
       </c>
       <c r="L11" s="32" t="inlineStr"/>
       <c r="M11" s="35" t="n">
@@ -2296,12 +2360,16 @@
       <c r="H12" s="42" t="n">
         <v>526699800</v>
       </c>
-      <c r="I12" s="39" t="inlineStr"/>
+      <c r="I12" s="39" t="inlineStr">
+        <is>
+          <t>127/QĐ-PCVT, ngày 30/03/2026</t>
+        </is>
+      </c>
       <c r="J12" s="42" t="n">
-        <v>0</v>
+        <v>523</v>
       </c>
       <c r="K12" s="42" t="n">
-        <v>527000000</v>
+        <v>440</v>
       </c>
       <c r="L12" s="39" t="inlineStr"/>
       <c r="M12" s="42" t="n">
@@ -2327,7 +2395,11 @@
       <c r="W12" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="X12" s="39" t="inlineStr"/>
+      <c r="X12" s="39" t="inlineStr">
+        <is>
+          <t>Công ty điện lực Vũng Tàu</t>
+        </is>
+      </c>
       <c r="Y12" s="39" t="inlineStr"/>
       <c r="Z12" s="43" t="n">
         <v>0</v>
@@ -2374,14 +2446,14 @@
       </c>
       <c r="I13" s="32" t="inlineStr"/>
       <c r="J13" s="35" t="n">
-        <v>0</v>
+        <v>18305</v>
       </c>
       <c r="K13" s="35" t="n">
-        <v>19016638310</v>
+        <v>14682</v>
       </c>
       <c r="L13" s="32" t="inlineStr"/>
       <c r="M13" s="35" t="n">
-        <v>0</v>
+        <v>18305</v>
       </c>
       <c r="N13" s="32" t="inlineStr"/>
       <c r="O13" s="35" t="n">
@@ -2389,11 +2461,11 @@
       </c>
       <c r="P13" s="32" t="inlineStr"/>
       <c r="Q13" s="35" t="n">
-        <v>0</v>
+        <v>4827</v>
       </c>
       <c r="R13" s="32" t="inlineStr"/>
       <c r="S13" s="35" t="n">
-        <v>0</v>
+        <v>4827</v>
       </c>
       <c r="T13" s="32" t="inlineStr"/>
       <c r="U13" s="35" t="n">
@@ -2462,16 +2534,24 @@
       <c r="H14" s="42" t="n">
         <v>13236612376</v>
       </c>
-      <c r="I14" s="39" t="inlineStr"/>
+      <c r="I14" s="39" t="inlineStr">
+        <is>
+          <t>108/QĐ-PCVT, ngày 30/03/2026</t>
+        </is>
+      </c>
       <c r="J14" s="42" t="n">
-        <v>0</v>
+        <v>13236</v>
       </c>
       <c r="K14" s="42" t="n">
-        <v>13236612376</v>
-      </c>
-      <c r="L14" s="39" t="inlineStr"/>
+        <v>10604</v>
+      </c>
+      <c r="L14" s="39" t="inlineStr">
+        <is>
+          <t>118/QĐ-PCVT</t>
+        </is>
+      </c>
       <c r="M14" s="42" t="n">
-        <v>0</v>
+        <v>13236</v>
       </c>
       <c r="N14" s="39" t="inlineStr"/>
       <c r="O14" s="42" t="n">
@@ -2493,7 +2573,11 @@
       <c r="W14" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="X14" s="39" t="inlineStr"/>
+      <c r="X14" s="39" t="inlineStr">
+        <is>
+          <t>Công ty điện lực Vũng Tàu</t>
+        </is>
+      </c>
       <c r="Y14" s="39" t="inlineStr"/>
       <c r="Z14" s="43" t="n">
         <v>0</v>
@@ -2565,16 +2649,24 @@
       <c r="H15" s="42" t="n">
         <v>5780025934</v>
       </c>
-      <c r="I15" s="39" t="inlineStr"/>
+      <c r="I15" s="39" t="inlineStr">
+        <is>
+          <t>128/QĐ-PCVT, ngày 13/03/2026</t>
+        </is>
+      </c>
       <c r="J15" s="42" t="n">
-        <v>0</v>
+        <v>5069</v>
       </c>
       <c r="K15" s="42" t="n">
-        <v>5780025934</v>
-      </c>
-      <c r="L15" s="39" t="inlineStr"/>
+        <v>4078</v>
+      </c>
+      <c r="L15" s="39" t="inlineStr">
+        <is>
+          <t>160/QĐ-PCVT</t>
+        </is>
+      </c>
       <c r="M15" s="42" t="n">
-        <v>0</v>
+        <v>5069</v>
       </c>
       <c r="N15" s="39" t="inlineStr"/>
       <c r="O15" s="42" t="n">
@@ -2582,11 +2674,15 @@
       </c>
       <c r="P15" s="39" t="inlineStr"/>
       <c r="Q15" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="39" t="inlineStr"/>
+        <v>4827</v>
+      </c>
+      <c r="R15" s="39" t="inlineStr">
+        <is>
+          <t>1314/HĐ-PCVT</t>
+        </is>
+      </c>
       <c r="S15" s="42" t="n">
-        <v>0</v>
+        <v>4827</v>
       </c>
       <c r="T15" s="39" t="inlineStr"/>
       <c r="U15" s="42" t="n">
@@ -2596,8 +2692,16 @@
       <c r="W15" s="42" t="n">
         <v>0</v>
       </c>
-      <c r="X15" s="39" t="inlineStr"/>
-      <c r="Y15" s="39" t="inlineStr"/>
+      <c r="X15" s="39" t="inlineStr">
+        <is>
+          <t>CHI NHÁNH TỔNG CÔNG TY ĐIỆN LỰC TPHCM TNHH – CÔNG TY DỊCH VỤ ĐIỆN LỰC TPHCM</t>
+        </is>
+      </c>
+      <c r="Y15" s="39" t="inlineStr">
+        <is>
+          <t>29/03/2026</t>
+        </is>
+      </c>
       <c r="Z15" s="43" t="n">
         <v>0</v>
       </c>
@@ -2643,26 +2747,26 @@
       </c>
       <c r="I16" s="32" t="inlineStr"/>
       <c r="J16" s="35" t="n">
-        <v>0</v>
+        <v>3311666745</v>
       </c>
       <c r="K16" s="35" t="n">
-        <v>37453293637</v>
+        <v>40475</v>
       </c>
       <c r="L16" s="32" t="inlineStr"/>
       <c r="M16" s="35" t="n">
-        <v>0</v>
+        <v>32217</v>
       </c>
       <c r="N16" s="32" t="inlineStr"/>
       <c r="O16" s="35" t="n">
-        <v>0</v>
+        <v>11705</v>
       </c>
       <c r="P16" s="32" t="inlineStr"/>
       <c r="Q16" s="35" t="n">
-        <v>11333808687</v>
+        <v>16607</v>
       </c>
       <c r="R16" s="32" t="inlineStr"/>
       <c r="S16" s="35" t="n">
-        <v>0</v>
+        <v>16607</v>
       </c>
       <c r="T16" s="32" t="inlineStr"/>
       <c r="U16" s="35" t="n">

</xml_diff>